<commit_message>
Fill in 264435 length/size; keep totals row as the last row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdaswSYFcee6fKLManU3ri
</commit_message>
<xml_diff>
--- a/deliverables/Khloe_VHS_Digitization_Log.xlsx
+++ b/deliverables/Khloe_VHS_Digitization_Log.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Tape Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tape Log'!$A$4:$F$37</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tape Log'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tape Log'!$A$9:$F$42</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tape Log'!$9:$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,27 +101,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="46" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="46" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="46" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="46" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -204,27 +202,17 @@
     <author>Claude</author>
   </authors>
   <commentList>
-    <comment ref="E6" authorId="0" shapeId="0">
-      <text>
-        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
-      </text>
-    </comment>
-    <comment ref="E9" authorId="0" shapeId="0">
-      <text>
-        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
-      </text>
-    </comment>
     <comment ref="E10" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E12" authorId="0" shapeId="0">
-      <text>
-        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
-      </text>
-    </comment>
-    <comment ref="E13" authorId="0" shapeId="0">
+    <comment ref="E11" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
+    <comment ref="E14" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
@@ -234,11 +222,6 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E16" authorId="0" shapeId="0">
-      <text>
-        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
-      </text>
-    </comment>
     <comment ref="E17" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
@@ -249,11 +232,6 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E19" authorId="0" shapeId="0">
-      <text>
-        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
-      </text>
-    </comment>
     <comment ref="E20" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
@@ -279,12 +257,37 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
+    <comment ref="E25" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
     <comment ref="E26" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
+    <comment ref="E27" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
     <comment ref="E28" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
+    <comment ref="E29" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
+    <comment ref="E31" authorId="0" shapeId="0">
+      <text>
+        <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
+      </text>
+    </comment>
+    <comment ref="E33" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
@@ -582,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -607,663 +610,674 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Yellow cells = to be filled in (descriptions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Size (GB) is calculated from File Size (KB) ÷ 1,048,576 — matches the GB figure Windows displays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Cells with a red corner comment: last digit of KB value was cut off in the screenshot (error &lt; 10 KB).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Barcodes 264529 and 264535 do not appear in the file list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL row at the bottom sums all running time and file sizes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Barcode #</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Length</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Size (GB)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>File Size (KB)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>264435</v>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7">
-        <f>IF(E5="","",E5/1048576)</f>
-        <v/>
-      </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>Length pending; File size pending; Out of sequence – possibly meant to be 264535 (missing from list)? Verify barcode.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8" t="n">
+        <v>0.2268287037037037</v>
+      </c>
+      <c r="D10" s="9">
+        <f>IF(E10="","",E10/1048576)</f>
+        <v/>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>295799070</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Out of sequence – possibly meant to be 264535 (missing from list)? Verify barcode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
         <v>264522</v>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="10" t="n">
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="8" t="n">
         <v>0.08130787037037036</v>
       </c>
-      <c r="D6" s="7">
-        <f>IF(E6="","",E6/1048576)</f>
-        <v/>
-      </c>
-      <c r="E6" s="11" t="n">
+      <c r="D11" s="9">
+        <f>IF(E11="","",E11/1048576)</f>
+        <v/>
+      </c>
+      <c r="E11" s="10" t="n">
         <v>104339010</v>
       </c>
-      <c r="F6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="F11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>264523</v>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="10" t="n">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="8" t="n">
         <v>0.03144675925925926</v>
       </c>
-      <c r="D7" s="7">
-        <f>IF(E7="","",E7/1048576)</f>
-        <v/>
-      </c>
-      <c r="E7" s="11" t="n">
+      <c r="D12" s="9">
+        <f>IF(E12="","",E12/1048576)</f>
+        <v/>
+      </c>
+      <c r="E12" s="10" t="n">
         <v>41343940</v>
       </c>
-      <c r="F7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="F12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
         <v>264524</v>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="10" t="n">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="8" t="n">
         <v>0.004085648148148148</v>
       </c>
-      <c r="D8" s="7">
-        <f>IF(E8="","",E8/1048576)</f>
-        <v/>
-      </c>
-      <c r="E8" s="11" t="n">
+      <c r="D13" s="9">
+        <f>IF(E13="","",E13/1048576)</f>
+        <v/>
+      </c>
+      <c r="E13" s="10" t="n">
         <v>5303859</v>
       </c>
-      <c r="F8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="F13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>264525</v>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="10" t="n">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="8" t="n">
         <v>0.08260416666666667</v>
       </c>
-      <c r="D9" s="7">
-        <f>IF(E9="","",E9/1048576)</f>
-        <v/>
-      </c>
-      <c r="E9" s="11" t="n">
+      <c r="D14" s="9">
+        <f>IF(E14="","",E14/1048576)</f>
+        <v/>
+      </c>
+      <c r="E14" s="10" t="n">
         <v>107631480</v>
       </c>
-      <c r="F9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
         <v>264526</v>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="10" t="n">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="8" t="n">
         <v>0.1256944444444444</v>
       </c>
-      <c r="D10" s="7">
-        <f>IF(E10="","",E10/1048576)</f>
-        <v/>
-      </c>
-      <c r="E10" s="11" t="n">
+      <c r="D15" s="9">
+        <f>IF(E15="","",E15/1048576)</f>
+        <v/>
+      </c>
+      <c r="E15" s="10" t="n">
         <v>164086750</v>
       </c>
-      <c r="F10" s="9" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="F15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>264527</v>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="10" t="n">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="8" t="n">
         <v>0.04659722222222222</v>
       </c>
-      <c r="D11" s="7">
-        <f>IF(E11="","",E11/1048576)</f>
-        <v/>
-      </c>
-      <c r="E11" s="11" t="n">
+      <c r="D16" s="9">
+        <f>IF(E16="","",E16/1048576)</f>
+        <v/>
+      </c>
+      <c r="E16" s="10" t="n">
         <v>60802001</v>
       </c>
-      <c r="F11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="F16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>264528</v>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="10" t="n">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="8" t="n">
         <v>0.08125</v>
       </c>
-      <c r="D12" s="7">
-        <f>IF(E12="","",E12/1048576)</f>
-        <v/>
-      </c>
-      <c r="E12" s="11" t="n">
+      <c r="D17" s="9">
+        <f>IF(E17="","",E17/1048576)</f>
+        <v/>
+      </c>
+      <c r="E17" s="10" t="n">
         <v>105659550</v>
       </c>
-      <c r="F12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="F17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>264530</v>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="10" t="n">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="8" t="n">
         <v>0.0880787037037037</v>
       </c>
-      <c r="D13" s="7">
-        <f>IF(E13="","",E13/1048576)</f>
-        <v/>
-      </c>
-      <c r="E13" s="11" t="n">
+      <c r="D18" s="9">
+        <f>IF(E18="","",E18/1048576)</f>
+        <v/>
+      </c>
+      <c r="E18" s="10" t="n">
         <v>116554860</v>
       </c>
-      <c r="F13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="F18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
         <v>264531</v>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="10" t="n">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="8" t="n">
         <v>0.003263888888888889</v>
       </c>
-      <c r="D14" s="7">
-        <f>IF(E14="","",E14/1048576)</f>
-        <v/>
-      </c>
-      <c r="E14" s="11" t="n">
+      <c r="D19" s="9">
+        <f>IF(E19="","",E19/1048576)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10" t="n">
         <v>4271085</v>
       </c>
-      <c r="F14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="F19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
         <v>264532</v>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="10" t="n">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="8" t="n">
         <v>0.09322916666666667</v>
       </c>
-      <c r="D15" s="7">
-        <f>IF(E15="","",E15/1048576)</f>
-        <v/>
-      </c>
-      <c r="E15" s="11" t="n">
+      <c r="D20" s="9">
+        <f>IF(E20="","",E20/1048576)</f>
+        <v/>
+      </c>
+      <c r="E20" s="10" t="n">
         <v>111412750</v>
       </c>
-      <c r="F15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="F20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
         <v>264533</v>
       </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="10" t="n">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="8" t="n">
         <v>0.2581018518518519</v>
       </c>
-      <c r="D16" s="7">
-        <f>IF(E16="","",E16/1048576)</f>
-        <v/>
-      </c>
-      <c r="E16" s="11" t="n">
+      <c r="D21" s="9">
+        <f>IF(E21="","",E21/1048576)</f>
+        <v/>
+      </c>
+      <c r="E21" s="10" t="n">
         <v>336680130</v>
       </c>
-      <c r="F16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="F21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
         <v>264534</v>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="10" t="n">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="8" t="n">
         <v>0.200787037037037</v>
       </c>
-      <c r="D17" s="7">
-        <f>IF(E17="","",E17/1048576)</f>
-        <v/>
-      </c>
-      <c r="E17" s="11" t="n">
+      <c r="D22" s="9">
+        <f>IF(E22="","",E22/1048576)</f>
+        <v/>
+      </c>
+      <c r="E22" s="10" t="n">
         <v>261374190</v>
       </c>
-      <c r="F17" s="9" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="F22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
         <v>264536</v>
       </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="10" t="n">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="8" t="n">
         <v>0.1615740740740741</v>
       </c>
-      <c r="D18" s="7">
-        <f>IF(E18="","",E18/1048576)</f>
-        <v/>
-      </c>
-      <c r="E18" s="11" t="n">
+      <c r="D23" s="9">
+        <f>IF(E23="","",E23/1048576)</f>
+        <v/>
+      </c>
+      <c r="E23" s="10" t="n">
         <v>211604860</v>
       </c>
-      <c r="F18" s="9" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="F23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
         <v>264537</v>
       </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="10" t="n">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="8" t="n">
         <v>0.1662037037037037</v>
       </c>
-      <c r="D19" s="7">
-        <f>IF(E19="","",E19/1048576)</f>
-        <v/>
-      </c>
-      <c r="E19" s="11" t="n">
+      <c r="D24" s="9">
+        <f>IF(E24="","",E24/1048576)</f>
+        <v/>
+      </c>
+      <c r="E24" s="10" t="n">
         <v>216744800</v>
       </c>
-      <c r="F19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="F24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
         <v>264538</v>
       </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="10" t="n">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="8" t="n">
         <v>0.1738194444444444</v>
       </c>
-      <c r="D20" s="7">
-        <f>IF(E20="","",E20/1048576)</f>
-        <v/>
-      </c>
-      <c r="E20" s="11" t="n">
+      <c r="D25" s="9">
+        <f>IF(E25="","",E25/1048576)</f>
+        <v/>
+      </c>
+      <c r="E25" s="10" t="n">
         <v>227090670</v>
       </c>
-      <c r="F20" s="9" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="F25" s="11" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
         <v>264539</v>
       </c>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="10" t="n">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="8" t="n">
         <v>0.1583796296296296</v>
       </c>
-      <c r="D21" s="7">
-        <f>IF(E21="","",E21/1048576)</f>
-        <v/>
-      </c>
-      <c r="E21" s="11" t="n">
+      <c r="D26" s="9">
+        <f>IF(E26="","",E26/1048576)</f>
+        <v/>
+      </c>
+      <c r="E26" s="10" t="n">
         <v>204842580</v>
       </c>
-      <c r="F21" s="9" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="F26" s="11" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
         <v>264540</v>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="10" t="n">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="8" t="n">
         <v>0.1038773148148148</v>
       </c>
-      <c r="D22" s="7">
-        <f>IF(E22="","",E22/1048576)</f>
-        <v/>
-      </c>
-      <c r="E22" s="11" t="n">
+      <c r="D27" s="9">
+        <f>IF(E27="","",E27/1048576)</f>
+        <v/>
+      </c>
+      <c r="E27" s="10" t="n">
         <v>134207210</v>
       </c>
-      <c r="F22" s="9" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="F27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
         <v>264541</v>
       </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="10" t="n">
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="8" t="n">
         <v>0.2556597222222222</v>
       </c>
-      <c r="D23" s="7">
-        <f>IF(E23="","",E23/1048576)</f>
-        <v/>
-      </c>
-      <c r="E23" s="11" t="n">
+      <c r="D28" s="9">
+        <f>IF(E28="","",E28/1048576)</f>
+        <v/>
+      </c>
+      <c r="E28" s="10" t="n">
         <v>332573120</v>
       </c>
-      <c r="F23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="F28" s="11" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
         <v>264542</v>
       </c>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="10" t="n">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="8" t="n">
         <v>0.1752546296296296</v>
       </c>
-      <c r="D24" s="7">
-        <f>IF(E24="","",E24/1048576)</f>
-        <v/>
-      </c>
-      <c r="E24" s="11" t="n">
+      <c r="D29" s="9">
+        <f>IF(E29="","",E29/1048576)</f>
+        <v/>
+      </c>
+      <c r="E29" s="10" t="n">
         <v>232685580</v>
       </c>
-      <c r="F24" s="9" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="F29" s="11" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
         <v>264543</v>
       </c>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="10" t="n">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="8" t="n">
         <v>0.002418981481481482</v>
       </c>
-      <c r="D25" s="7">
-        <f>IF(E25="","",E25/1048576)</f>
-        <v/>
-      </c>
-      <c r="E25" s="11" t="n">
+      <c r="D30" s="9">
+        <f>IF(E30="","",E30/1048576)</f>
+        <v/>
+      </c>
+      <c r="E30" s="10" t="n">
         <v>3255693</v>
       </c>
-      <c r="F25" s="9" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="F30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
         <v>264544</v>
       </c>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="10" t="n">
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="8" t="n">
         <v>0.08690972222222222</v>
       </c>
-      <c r="D26" s="7">
-        <f>IF(E26="","",E26/1048576)</f>
-        <v/>
-      </c>
-      <c r="E26" s="11" t="n">
+      <c r="D31" s="9">
+        <f>IF(E31="","",E31/1048576)</f>
+        <v/>
+      </c>
+      <c r="E31" s="10" t="n">
         <v>110644070</v>
       </c>
-      <c r="F26" s="9" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="F31" s="11" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
         <v>264545</v>
       </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="10" t="n">
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="8" t="n">
         <v>0.002488425925925926</v>
       </c>
-      <c r="D27" s="7">
-        <f>IF(E27="","",E27/1048576)</f>
-        <v/>
-      </c>
-      <c r="E27" s="11" t="n">
+      <c r="D32" s="9">
+        <f>IF(E32="","",E32/1048576)</f>
+        <v/>
+      </c>
+      <c r="E32" s="10" t="n">
         <v>3327299</v>
       </c>
-      <c r="F27" s="9" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="F32" s="11" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
         <v>264546</v>
       </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="10" t="n">
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="8" t="n">
         <v>0.08737268518518519</v>
       </c>
-      <c r="D28" s="7">
-        <f>IF(E28="","",E28/1048576)</f>
-        <v/>
-      </c>
-      <c r="E28" s="11" t="n">
+      <c r="D33" s="9">
+        <f>IF(E33="","",E33/1048576)</f>
+        <v/>
+      </c>
+      <c r="E33" s="10" t="n">
         <v>111408390</v>
       </c>
-      <c r="F28" s="9" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="F33" s="11" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
         <v>264547</v>
       </c>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="10" t="n">
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="8" t="n">
         <v>0.02819444444444445</v>
       </c>
-      <c r="D29" s="7">
-        <f>IF(E29="","",E29/1048576)</f>
-        <v/>
-      </c>
-      <c r="E29" s="11" t="n">
+      <c r="D34" s="9">
+        <f>IF(E34="","",E34/1048576)</f>
+        <v/>
+      </c>
+      <c r="E34" s="10" t="n">
         <v>36064668</v>
       </c>
-      <c r="F29" s="9" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="F34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
         <v>264548</v>
       </c>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="10" t="n">
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="8" t="n">
         <v>0.03559027777777778</v>
       </c>
-      <c r="D30" s="7">
-        <f>IF(E30="","",E30/1048576)</f>
-        <v/>
-      </c>
-      <c r="E30" s="11" t="n">
+      <c r="D35" s="9">
+        <f>IF(E35="","",E35/1048576)</f>
+        <v/>
+      </c>
+      <c r="E35" s="10" t="n">
         <v>46962994</v>
       </c>
-      <c r="F30" s="9" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="F35" s="11" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
         <v>264549</v>
       </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="10" t="n">
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="8" t="n">
         <v>0.07180555555555555</v>
       </c>
-      <c r="D31" s="7">
-        <f>IF(E31="","",E31/1048576)</f>
-        <v/>
-      </c>
-      <c r="E31" s="11" t="n">
+      <c r="D36" s="9">
+        <f>IF(E36="","",E36/1048576)</f>
+        <v/>
+      </c>
+      <c r="E36" s="10" t="n">
         <v>96787150</v>
       </c>
-      <c r="F31" s="9" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="F36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
         <v>264550</v>
       </c>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="10" t="n">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="8" t="n">
         <v>0.07075231481481481</v>
       </c>
-      <c r="D32" s="7">
-        <f>IF(E32="","",E32/1048576)</f>
-        <v/>
-      </c>
-      <c r="E32" s="11" t="n">
+      <c r="D37" s="9">
+        <f>IF(E37="","",E37/1048576)</f>
+        <v/>
+      </c>
+      <c r="E37" s="10" t="n">
         <v>95363950</v>
       </c>
-      <c r="F32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
         <v>264551</v>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="10" t="n">
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="8" t="n">
         <v>0.00974537037037037</v>
       </c>
-      <c r="D33" s="7">
-        <f>IF(E33="","",E33/1048576)</f>
-        <v/>
-      </c>
-      <c r="E33" s="11" t="n">
+      <c r="D38" s="9">
+        <f>IF(E38="","",E38/1048576)</f>
+        <v/>
+      </c>
+      <c r="E38" s="10" t="n">
         <v>13024655</v>
       </c>
-      <c r="F33" s="9" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="F38" s="11" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
         <v>264552</v>
       </c>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="10" t="n">
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="8" t="n">
         <v>0.02221064814814815</v>
       </c>
-      <c r="D34" s="7">
-        <f>IF(E34="","",E34/1048576)</f>
-        <v/>
-      </c>
-      <c r="E34" s="11" t="n">
+      <c r="D39" s="9">
+        <f>IF(E39="","",E39/1048576)</f>
+        <v/>
+      </c>
+      <c r="E39" s="10" t="n">
         <v>28722522</v>
       </c>
-      <c r="F34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="F39" s="11" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>264553</v>
       </c>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="10" t="n">
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="8" t="n">
         <v>0.04520833333333334</v>
       </c>
-      <c r="D35" s="7">
-        <f>IF(E35="","",E35/1048576)</f>
-        <v/>
-      </c>
-      <c r="E35" s="11" t="n">
+      <c r="D40" s="9">
+        <f>IF(E40="","",E40/1048576)</f>
+        <v/>
+      </c>
+      <c r="E40" s="10" t="n">
         <v>60265882</v>
       </c>
-      <c r="F35" s="9" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="F40" s="11" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>264554</v>
       </c>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="10" t="n">
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="8" t="n">
         <v>0.04619212962962963</v>
       </c>
-      <c r="D36" s="7">
-        <f>IF(E36="","",E36/1048576)</f>
-        <v/>
-      </c>
-      <c r="E36" s="11" t="n">
+      <c r="D41" s="9">
+        <f>IF(E41="","",E41/1048576)</f>
+        <v/>
+      </c>
+      <c r="E41" s="10" t="n">
         <v>60001573</v>
       </c>
-      <c r="F36" s="9" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="F41" s="11" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
         <v>264555</v>
       </c>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="10" t="n">
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="8" t="n">
         <v>0.04660879629629629</v>
       </c>
-      <c r="D37" s="7">
-        <f>IF(E37="","",E37/1048576)</f>
-        <v/>
-      </c>
-      <c r="E37" s="11" t="n">
+      <c r="D42" s="9">
+        <f>IF(E42="","",E42/1048576)</f>
+        <v/>
+      </c>
+      <c r="E42" s="10" t="n">
         <v>60869791</v>
       </c>
-      <c r="F37" s="9" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="F42" s="11" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B38" s="12">
-        <f>COUNTA(A5:A37)&amp;" tapes"</f>
-        <v/>
-      </c>
-      <c r="C38" s="13">
-        <f>SUM(C5:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="14">
-        <f>SUM(D5:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="15">
-        <f>SUM(E5:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="12">
-        <f>TEXT(D38/1024,"0.00")&amp;" TB total"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Legend:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t>Yellow cells = to be filled in (descriptions, and length/size for 264435).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>Size (GB) is calculated from File Size (KB) ÷ 1,048,576 — matches the GB figure Windows displays.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>Cells with a red corner comment: last digit of KB value was cut off in the screenshot (error &lt; 10 KB).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>Barcodes 264529 and 264535 do not appear in the file list.</t>
-        </is>
+      <c r="B43" s="12">
+        <f>COUNTA(A10:A42)&amp;" tapes"</f>
+        <v/>
+      </c>
+      <c r="C43" s="13">
+        <f>SUM(C10:C42)</f>
+        <v/>
+      </c>
+      <c r="D43" s="14">
+        <f>SUM(D10:D42)</f>
+        <v/>
+      </c>
+      <c r="E43" s="15">
+        <f>SUM(E10:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="12">
+        <f>TEXT(D43/1024,"0.00")&amp;" TB total"</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F37"/>
+  <autoFilter ref="A9:F42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Correct barcode 264435 to 264535 and sort into sequence
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdaswSYFcee6fKLManU3ri
</commit_message>
<xml_diff>
--- a/deliverables/Khloe_VHS_Digitization_Log.xlsx
+++ b/deliverables/Khloe_VHS_Digitization_Log.xlsx
@@ -207,7 +207,7 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E11" authorId="0" shapeId="0">
+    <comment ref="E13" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
@@ -217,7 +217,7 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E15" authorId="0" shapeId="0">
+    <comment ref="E16" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
@@ -227,7 +227,7 @@
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
     </comment>
-    <comment ref="E18" authorId="0" shapeId="0">
+    <comment ref="E19" authorId="0" shapeId="0">
       <text>
         <t>Last digit was cut off in Explorer; entered as 0 (off by &lt;10 KB). Replace with exact value if needed.</t>
       </text>
@@ -641,7 +641,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Barcodes 264529 and 264535 do not appear in the file list.</t>
+          <t>Barcode 264529 does not appear in the file list.</t>
         </is>
       </c>
     </row>
@@ -686,228 +686,228 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>264435</v>
+        <v>264522</v>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="8" t="n">
-        <v>0.2268287037037037</v>
+        <v>0.08130787037037036</v>
       </c>
       <c r="D10" s="9">
         <f>IF(E10="","",E10/1048576)</f>
         <v/>
       </c>
       <c r="E10" s="10" t="n">
-        <v>295799070</v>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Out of sequence – possibly meant to be 264535 (missing from list)? Verify barcode.</t>
-        </is>
-      </c>
+        <v>104339010</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>264522</v>
+        <v>264523</v>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="8" t="n">
-        <v>0.08130787037037036</v>
+        <v>0.03144675925925926</v>
       </c>
       <c r="D11" s="9">
         <f>IF(E11="","",E11/1048576)</f>
         <v/>
       </c>
       <c r="E11" s="10" t="n">
-        <v>104339010</v>
+        <v>41343940</v>
       </c>
       <c r="F11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>264523</v>
+        <v>264524</v>
       </c>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="8" t="n">
-        <v>0.03144675925925926</v>
+        <v>0.004085648148148148</v>
       </c>
       <c r="D12" s="9">
         <f>IF(E12="","",E12/1048576)</f>
         <v/>
       </c>
       <c r="E12" s="10" t="n">
-        <v>41343940</v>
+        <v>5303859</v>
       </c>
       <c r="F12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>264524</v>
+        <v>264525</v>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="8" t="n">
-        <v>0.004085648148148148</v>
+        <v>0.08260416666666667</v>
       </c>
       <c r="D13" s="9">
         <f>IF(E13="","",E13/1048576)</f>
         <v/>
       </c>
       <c r="E13" s="10" t="n">
-        <v>5303859</v>
+        <v>107631480</v>
       </c>
       <c r="F13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>264525</v>
+        <v>264526</v>
       </c>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="8" t="n">
-        <v>0.08260416666666667</v>
+        <v>0.1256944444444444</v>
       </c>
       <c r="D14" s="9">
         <f>IF(E14="","",E14/1048576)</f>
         <v/>
       </c>
       <c r="E14" s="10" t="n">
-        <v>107631480</v>
+        <v>164086750</v>
       </c>
       <c r="F14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>264526</v>
+        <v>264527</v>
       </c>
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="8" t="n">
-        <v>0.1256944444444444</v>
+        <v>0.04659722222222222</v>
       </c>
       <c r="D15" s="9">
         <f>IF(E15="","",E15/1048576)</f>
         <v/>
       </c>
       <c r="E15" s="10" t="n">
-        <v>164086750</v>
+        <v>60802001</v>
       </c>
       <c r="F15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>264527</v>
+        <v>264528</v>
       </c>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="8" t="n">
-        <v>0.04659722222222222</v>
+        <v>0.08125</v>
       </c>
       <c r="D16" s="9">
         <f>IF(E16="","",E16/1048576)</f>
         <v/>
       </c>
       <c r="E16" s="10" t="n">
-        <v>60802001</v>
+        <v>105659550</v>
       </c>
       <c r="F16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>264528</v>
+        <v>264530</v>
       </c>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="8" t="n">
-        <v>0.08125</v>
+        <v>0.0880787037037037</v>
       </c>
       <c r="D17" s="9">
         <f>IF(E17="","",E17/1048576)</f>
         <v/>
       </c>
       <c r="E17" s="10" t="n">
-        <v>105659550</v>
+        <v>116554860</v>
       </c>
       <c r="F17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>264530</v>
+        <v>264531</v>
       </c>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="8" t="n">
-        <v>0.0880787037037037</v>
+        <v>0.003263888888888889</v>
       </c>
       <c r="D18" s="9">
         <f>IF(E18="","",E18/1048576)</f>
         <v/>
       </c>
       <c r="E18" s="10" t="n">
-        <v>116554860</v>
+        <v>4271085</v>
       </c>
       <c r="F18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>264531</v>
+        <v>264532</v>
       </c>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="8" t="n">
-        <v>0.003263888888888889</v>
+        <v>0.09322916666666667</v>
       </c>
       <c r="D19" s="9">
         <f>IF(E19="","",E19/1048576)</f>
         <v/>
       </c>
       <c r="E19" s="10" t="n">
-        <v>4271085</v>
+        <v>111412750</v>
       </c>
       <c r="F19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>264532</v>
+        <v>264533</v>
       </c>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="8" t="n">
-        <v>0.09322916666666667</v>
+        <v>0.2581018518518519</v>
       </c>
       <c r="D20" s="9">
         <f>IF(E20="","",E20/1048576)</f>
         <v/>
       </c>
       <c r="E20" s="10" t="n">
-        <v>111412750</v>
+        <v>336680130</v>
       </c>
       <c r="F20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>264533</v>
+        <v>264534</v>
       </c>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="8" t="n">
-        <v>0.2581018518518519</v>
+        <v>0.200787037037037</v>
       </c>
       <c r="D21" s="9">
         <f>IF(E21="","",E21/1048576)</f>
         <v/>
       </c>
       <c r="E21" s="10" t="n">
-        <v>336680130</v>
+        <v>261374190</v>
       </c>
       <c r="F21" s="11" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>264534</v>
+        <v>264535</v>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="8" t="n">
-        <v>0.200787037037037</v>
+        <v>0.2268287037037037</v>
       </c>
       <c r="D22" s="9">
         <f>IF(E22="","",E22/1048576)</f>
         <v/>
       </c>
       <c r="E22" s="10" t="n">
-        <v>261374190</v>
-      </c>
-      <c r="F22" s="11" t="inlineStr"/>
+        <v>295799070</v>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>File currently misnamed 264435.mov on drive – rename to 264535.mov before delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">

</xml_diff>

<commit_message>
Note no audio on tape 264554
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdaswSYFcee6fKLManU3ri
</commit_message>
<xml_diff>
--- a/deliverables/Khloe_VHS_Digitization_Log.xlsx
+++ b/deliverables/Khloe_VHS_Digitization_Log.xlsx
@@ -620,7 +620,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Yellow cells = to be filled in (descriptions).</t>
+          <t>Description column (yellow) is left blank for the client to fill in.</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,11 @@
       <c r="E41" s="10" t="n">
         <v>60001573</v>
       </c>
-      <c r="F41" s="11" t="inlineStr"/>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>No audio on source tape.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">

</xml_diff>

<commit_message>
Remove rename note for 264535
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdaswSYFcee6fKLManU3ri
</commit_message>
<xml_diff>
--- a/deliverables/Khloe_VHS_Digitization_Log.xlsx
+++ b/deliverables/Khloe_VHS_Digitization_Log.xlsx
@@ -729,11 +729,7 @@
       <c r="D21" s="9" t="n">
         <v>282.1</v>
       </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>File currently misnamed 264435.mov on drive – rename to 264535.mov before delivery.</t>
-        </is>
-      </c>
+      <c r="E21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">

</xml_diff>